<commit_message>
Updates logic challenge spreadsheet
</commit_message>
<xml_diff>
--- a/10-logic-challanges/1-challange.xlsx
+++ b/10-logic-challanges/1-challange.xlsx
@@ -497,10 +497,7 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="D2" s="2">
-        <f>IF(AND(B2&gt;=70,C2="Sim"),"Aprovado",IF(OR(B2&gt;=70,C2="Sim"),"Lista de espera","Reprovado"))</f>
-        <v/>
-      </c>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -516,10 +513,7 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="D3" s="3">
-        <f>IF(AND(B3&gt;=70,C3="Sim"),"Aprovado",IF(OR(B3&gt;=70,C3="Sim"),"Lista de espera","Reprovado"))</f>
-        <v/>
-      </c>
+      <c r="D3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -535,10 +529,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="D4" s="2">
-        <f>IF(AND(B4&gt;=70,C4="Sim"),"Aprovado",IF(OR(B4&gt;=70,C4="Sim"),"Lista de espera","Reprovado"))</f>
-        <v/>
-      </c>
+      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -554,10 +545,7 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="D5" s="3">
-        <f>IF(AND(B5&gt;=70,C5="Sim"),"Aprovado",IF(OR(B5&gt;=70,C5="Sim"),"Lista de espera","Reprovado"))</f>
-        <v/>
-      </c>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -573,10 +561,7 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="D6" s="2">
-        <f>IF(AND(B6&gt;=70,C6="Sim"),"Aprovado",IF(OR(B6&gt;=70,C6="Sim"),"Lista de espera","Reprovado"))</f>
-        <v/>
-      </c>
+      <c r="D6" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>